<commit_message>
updated sept 18 meet
</commit_message>
<xml_diff>
--- a/Meeting_Attendance.xlsx
+++ b/Meeting_Attendance.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="138">
   <si>
     <t>Name</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>Meeting 2026-09-11</t>
+  </si>
+  <si>
+    <t>Meeting 2026-09-18</t>
   </si>
   <si>
     <t>Ved Mewada</t>
@@ -782,10 +785,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -810,22 +813,25 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C2">
         <v>9998667888</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -836,22 +842,25 @@
       <c r="H2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:8">
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C3">
         <v>8467095435</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -862,22 +871,25 @@
       <c r="H3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:8">
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4">
         <v>7357511041</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -888,22 +900,25 @@
       <c r="H4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:8">
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5">
         <v>9177202100</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -914,22 +929,25 @@
       <c r="H5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:8">
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C6">
         <v>7395927689</v>
       </c>
       <c r="D6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -940,22 +958,25 @@
       <c r="H6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:8">
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C7">
         <v>7870068838</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -966,22 +987,25 @@
       <c r="H7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:8">
+      <c r="I7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C8">
         <v>8240087955</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -992,22 +1016,25 @@
       <c r="H8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:8">
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C9">
         <v>7603913238</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -1018,22 +1045,25 @@
       <c r="H9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:8">
+      <c r="I9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C10">
         <v>9884464562</v>
       </c>
       <c r="D10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -1044,22 +1074,25 @@
       <c r="H10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:8">
+      <c r="I10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C11">
         <v>9030730696</v>
       </c>
       <c r="D11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -1070,22 +1103,25 @@
       <c r="H11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:8">
+      <c r="I11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C12">
         <v>6372111245</v>
       </c>
       <c r="D12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -1096,22 +1132,25 @@
       <c r="H12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:8">
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C13">
         <v>7386723779</v>
       </c>
       <c r="D13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -1122,22 +1161,25 @@
       <c r="H13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:8">
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C14">
         <v>7006933519</v>
       </c>
       <c r="D14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -1148,22 +1190,25 @@
       <c r="H14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:8">
+      <c r="I14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C15">
         <v>9935712711</v>
       </c>
       <c r="D15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1174,22 +1219,25 @@
       <c r="H15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:8">
+      <c r="I15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C16">
         <v>9003223034</v>
       </c>
       <c r="D16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -1200,22 +1248,25 @@
       <c r="H16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:8">
+      <c r="I16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C17">
         <v>8950799910</v>
       </c>
       <c r="D17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1226,22 +1277,25 @@
       <c r="H17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:8">
+      <c r="I17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C18">
         <v>9398172990</v>
       </c>
       <c r="D18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E18" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -1252,22 +1306,25 @@
       <c r="H18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:8">
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C19">
         <v>9895297289</v>
       </c>
       <c r="D19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E19" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -1278,22 +1335,25 @@
       <c r="H19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:8">
+      <c r="I19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C20">
         <v>9399234486</v>
       </c>
       <c r="D20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E20" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -1304,22 +1364,25 @@
       <c r="H20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:8">
+      <c r="I20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C21">
         <v>8390904936</v>
       </c>
       <c r="D21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E21" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F21">
         <v>1</v>
@@ -1330,22 +1393,25 @@
       <c r="H21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:8">
+      <c r="I21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C22">
         <v>9025580044</v>
       </c>
       <c r="D22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1356,22 +1422,25 @@
       <c r="H22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:8">
+      <c r="I22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C23">
         <v>8718946895</v>
       </c>
       <c r="D23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1382,22 +1451,25 @@
       <c r="H23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:8">
+      <c r="I23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C24">
         <v>7305542772</v>
       </c>
       <c r="D24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E24" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1408,22 +1480,25 @@
       <c r="H24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:8">
+      <c r="I24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C25">
         <v>9655635923</v>
       </c>
       <c r="D25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E25" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1434,22 +1509,25 @@
       <c r="H25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:8">
+      <c r="I25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C26">
         <v>6301777824</v>
       </c>
       <c r="D26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E26" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1460,22 +1538,25 @@
       <c r="H26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:8">
+      <c r="I26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C27">
         <v>956211707</v>
       </c>
       <c r="D27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1486,22 +1567,25 @@
       <c r="H27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:8">
+      <c r="I27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C28">
         <v>7017097553</v>
       </c>
       <c r="D28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E28" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -1512,22 +1596,25 @@
       <c r="H28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:8">
+      <c r="I28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C29">
         <v>8547224301</v>
       </c>
       <c r="D29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F29">
         <v>1</v>
@@ -1538,22 +1625,25 @@
       <c r="H29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:8">
+      <c r="I29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C30">
         <v>9998667888</v>
       </c>
       <c r="D30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E30" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F30">
         <v>0</v>
@@ -1564,22 +1654,25 @@
       <c r="H30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:8">
+      <c r="I30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C31">
         <v>6379553392</v>
       </c>
       <c r="D31" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E31" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F31">
         <v>1</v>
@@ -1590,22 +1683,25 @@
       <c r="H31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:8">
+      <c r="I31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C32">
         <v>7877984342</v>
       </c>
       <c r="D32" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F32">
         <v>0</v>
@@ -1616,22 +1712,25 @@
       <c r="H32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:8">
+      <c r="I32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C33">
         <v>8369179576</v>
       </c>
       <c r="D33" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E33" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F33">
         <v>0</v>
@@ -1642,22 +1741,25 @@
       <c r="H33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:8">
+      <c r="I33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B34" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C34">
         <v>8075327997</v>
       </c>
       <c r="D34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -1668,22 +1770,25 @@
       <c r="H34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:8">
+      <c r="I34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
       <c r="A35" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B35" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C35">
         <v>9482712848</v>
       </c>
       <c r="D35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F35">
         <v>0</v>
@@ -1694,22 +1799,25 @@
       <c r="H35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:8">
+      <c r="I35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B36" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C36">
         <v>9500365662</v>
       </c>
       <c r="D36" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E36" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F36">
         <v>0</v>
@@ -1720,22 +1828,25 @@
       <c r="H36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:8">
+      <c r="I36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C37">
         <v>9840502912</v>
       </c>
       <c r="D37" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E37" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F37">
         <v>1</v>
@@ -1746,22 +1857,25 @@
       <c r="H37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:8">
+      <c r="I37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C38">
         <v>9884198689</v>
       </c>
       <c r="D38" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F38">
         <v>0</v>
@@ -1772,22 +1886,25 @@
       <c r="H38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:8">
+      <c r="I38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
       <c r="A39" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C39">
         <v>7606996818</v>
       </c>
       <c r="D39" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F39">
         <v>0</v>
@@ -1798,22 +1915,25 @@
       <c r="H39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:8">
+      <c r="I39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B40" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C40">
         <v>7013522537</v>
       </c>
       <c r="D40" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -1824,22 +1944,25 @@
       <c r="H40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:8">
+      <c r="I40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
       <c r="A41" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C41">
         <v>9734187783</v>
       </c>
       <c r="D41" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F41">
         <v>0</v>
@@ -1850,22 +1973,25 @@
       <c r="H41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:8">
+      <c r="I41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
       <c r="A42" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C42">
         <v>9361201097</v>
       </c>
       <c r="D42" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F42">
         <v>0</v>
@@ -1876,22 +2002,25 @@
       <c r="H42">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="1:8">
+      <c r="I42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
       <c r="A43" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C43">
         <v>9150943024</v>
       </c>
       <c r="D43" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F43">
         <v>0</v>
@@ -1902,22 +2031,25 @@
       <c r="H43">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:8">
+      <c r="I43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
       <c r="A44" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B44" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C44">
         <v>8637447960</v>
       </c>
       <c r="D44" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F44">
         <v>1</v>
@@ -1928,22 +2060,25 @@
       <c r="H44">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:8">
+      <c r="I44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
       <c r="A45" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C45">
         <v>9042769165</v>
       </c>
       <c r="D45" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E45" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F45">
         <v>0</v>
@@ -1952,6 +2087,9 @@
         <v>0</v>
       </c>
       <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated sept 18 meet again because ppl joined late
</commit_message>
<xml_diff>
--- a/Meeting_Attendance.xlsx
+++ b/Meeting_Attendance.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC contest tracking basic\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC65958F-8D5C-4ACC-8CF0-889587BDD7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -433,8 +439,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -497,13 +503,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -541,7 +555,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -575,6 +589,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -609,9 +624,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -784,11 +800,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I45"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.90625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -817,7 +836,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -846,7 +865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -875,7 +894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -904,7 +923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -933,7 +952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -962,7 +981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -991,7 +1010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1020,7 +1039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1049,7 +1068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -1078,7 +1097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -1107,7 +1126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1136,7 +1155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -1165,7 +1184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1194,7 +1213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1223,7 +1242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -1252,7 +1271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -1281,7 +1300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -1310,7 +1329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -1339,7 +1358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -1368,7 +1387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -1397,7 +1416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -1426,7 +1445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -1455,7 +1474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -1484,7 +1503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -1513,7 +1532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>33</v>
       </c>
@@ -1542,7 +1561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -1571,7 +1590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>35</v>
       </c>
@@ -1600,7 +1619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -1629,7 +1648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -1658,7 +1677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -1687,7 +1706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -1713,10 +1732,10 @@
         <v>1</v>
       </c>
       <c r="I32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>39</v>
       </c>
@@ -1745,7 +1764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -1774,7 +1793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>41</v>
       </c>
@@ -1803,7 +1822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -1832,7 +1851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -1861,7 +1880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>44</v>
       </c>
@@ -1890,7 +1909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>45</v>
       </c>
@@ -1919,7 +1938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>46</v>
       </c>
@@ -1948,7 +1967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -1977,7 +1996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -2003,10 +2022,10 @@
         <v>1</v>
       </c>
       <c r="I42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>49</v>
       </c>
@@ -2035,7 +2054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>50</v>
       </c>
@@ -2064,7 +2083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>51</v>
       </c>

</xml_diff>